<commit_message>
Added CO-PO-PSO Mapping in Capstone Project Sheet
</commit_message>
<xml_diff>
--- a/Attainment Calculation/Sheet from BRC for Attainment Calculation/CR 3_SEMINAR AND PROJECT INITIATION COURSE(315003).xlsx
+++ b/Attainment Calculation/Sheet from BRC for Attainment Calculation/CR 3_SEMINAR AND PROJECT INITIATION COURSE(315003).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MSBTE-28\Documents\ada\gpd_nba\Attainment Calculation\Sheet from BRC for Attainment Calculation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B3CD1BE-8652-4EF5-B4CE-682DC17512E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6B22095-4034-491C-BD00-5181BC8434A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PO Set Target attain level" sheetId="1" r:id="rId1"/>
@@ -3031,10 +3031,55 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3051,65 +3096,42 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="3" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="5" fillId="3" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3138,43 +3160,6 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3183,16 +3168,48 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="68" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="23" fillId="3" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3205,22 +3222,14 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="68" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="23" fillId="3" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3232,9 +3241,23 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="76" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="77" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3252,28 +3275,32 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="76" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="77" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="13" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3294,40 +3321,25 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="3" fillId="3" borderId="48" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="83" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="85" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="84" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="86" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3351,35 +3363,23 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="83" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="85" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="84" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="86" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="3" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="3" fillId="3" borderId="48" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4098,40 +4098,40 @@
       <c r="C3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="210" t="s">
+      <c r="D3" s="189" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="203"/>
+      <c r="E3" s="190"/>
     </row>
     <row r="4" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B4" s="6"/>
       <c r="C4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="210">
+      <c r="D4" s="189">
         <v>315003</v>
       </c>
-      <c r="E4" s="203"/>
+      <c r="E4" s="190"/>
     </row>
     <row r="5" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B5" s="4"/>
       <c r="C5" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="211" t="s">
+      <c r="D5" s="191" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="202"/>
+      <c r="E5" s="192"/>
     </row>
     <row r="6" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B6" s="4"/>
       <c r="C6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="210" t="s">
+      <c r="D6" s="189" t="s">
         <v>7</v>
       </c>
-      <c r="E6" s="203"/>
+      <c r="E6" s="190"/>
     </row>
     <row r="7" spans="2:13" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B7" s="7" t="s">
@@ -4146,50 +4146,50 @@
       <c r="C8" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="184" t="s">
+      <c r="D8" s="187" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="185"/>
+      <c r="E8" s="188"/>
     </row>
     <row r="9" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="6"/>
       <c r="C9" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="184" t="s">
+      <c r="D9" s="187" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="185"/>
+      <c r="E9" s="188"/>
     </row>
     <row r="10" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="6"/>
       <c r="C10" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="D10" s="184" t="s">
+      <c r="D10" s="187" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="185"/>
+      <c r="E10" s="188"/>
     </row>
     <row r="11" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="6"/>
       <c r="C11" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="D11" s="184" t="s">
+      <c r="D11" s="187" t="s">
         <v>16</v>
       </c>
-      <c r="E11" s="185"/>
+      <c r="E11" s="188"/>
     </row>
     <row r="12" spans="2:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="6"/>
       <c r="C12" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="184" t="s">
+      <c r="D12" s="187" t="s">
         <v>18</v>
       </c>
-      <c r="E12" s="185"/>
+      <c r="E12" s="188"/>
     </row>
     <row r="14" spans="2:13" ht="18.75" x14ac:dyDescent="0.25">
       <c r="B14" s="9" t="s">
@@ -4224,14 +4224,14 @@
       <c r="M15" s="11"/>
     </row>
     <row r="16" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B16" s="186" t="s">
+      <c r="B16" s="205" t="s">
         <v>21</v>
       </c>
-      <c r="C16" s="189" t="s">
+      <c r="C16" s="208" t="s">
         <v>22</v>
       </c>
-      <c r="D16" s="190"/>
-      <c r="E16" s="195" t="s">
+      <c r="D16" s="209"/>
+      <c r="E16" s="214" t="s">
         <v>23</v>
       </c>
       <c r="F16" s="196"/>
@@ -4239,16 +4239,16 @@
       <c r="H16" s="196"/>
       <c r="I16" s="196"/>
       <c r="J16" s="196"/>
-      <c r="K16" s="197"/>
-      <c r="L16" s="198" t="s">
+      <c r="K16" s="194"/>
+      <c r="L16" s="193" t="s">
         <v>24</v>
       </c>
-      <c r="M16" s="197"/>
+      <c r="M16" s="194"/>
     </row>
     <row r="17" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="B17" s="187"/>
-      <c r="C17" s="191"/>
-      <c r="D17" s="192"/>
+      <c r="B17" s="206"/>
+      <c r="C17" s="210"/>
+      <c r="D17" s="211"/>
       <c r="E17" s="13" t="s">
         <v>25</v>
       </c>
@@ -4278,9 +4278,9 @@
       </c>
     </row>
     <row r="18" spans="1:25" ht="122.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="188"/>
-      <c r="C18" s="193"/>
-      <c r="D18" s="194"/>
+      <c r="B18" s="207"/>
+      <c r="C18" s="212"/>
+      <c r="D18" s="213"/>
       <c r="E18" s="15" t="s">
         <v>34</v>
       </c>
@@ -4510,11 +4510,11 @@
       </c>
     </row>
     <row r="24" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="199" t="s">
+      <c r="B24" s="195" t="s">
         <v>44</v>
       </c>
       <c r="C24" s="196"/>
-      <c r="D24" s="197"/>
+      <c r="D24" s="194"/>
       <c r="E24" s="18">
         <f t="shared" ref="E24:K24" si="5">IFERROR(AVERAGE(E19:E23),2)</f>
         <v>2.6</v>
@@ -4553,11 +4553,11 @@
       </c>
     </row>
     <row r="25" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="200" t="s">
+      <c r="B25" s="197" t="s">
         <v>45</v>
       </c>
       <c r="C25" s="196"/>
-      <c r="D25" s="197"/>
+      <c r="D25" s="194"/>
       <c r="E25" s="24">
         <f t="shared" ref="E25:M25" si="7">E24</f>
         <v>2.6</v>
@@ -4601,32 +4601,32 @@
       <c r="D28" s="27" t="s">
         <v>250</v>
       </c>
-      <c r="I28" s="209" t="s">
+      <c r="I28" s="204" t="s">
         <v>46</v>
       </c>
-      <c r="J28" s="207"/>
-      <c r="K28" s="207"/>
-      <c r="L28" s="207"/>
-      <c r="M28" s="207"/>
+      <c r="J28" s="202"/>
+      <c r="K28" s="202"/>
+      <c r="L28" s="202"/>
+      <c r="M28" s="202"/>
     </row>
     <row r="29" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="28"/>
       <c r="B29" s="28"/>
-      <c r="C29" s="201" t="s">
+      <c r="C29" s="198" t="s">
         <v>47</v>
       </c>
-      <c r="D29" s="202"/>
-      <c r="E29" s="203"/>
+      <c r="D29" s="192"/>
+      <c r="E29" s="190"/>
       <c r="F29" s="28"/>
       <c r="G29" s="28"/>
       <c r="H29" s="28"/>
-      <c r="I29" s="201" t="s">
+      <c r="I29" s="198" t="s">
         <v>47</v>
       </c>
-      <c r="J29" s="202"/>
-      <c r="K29" s="202"/>
-      <c r="L29" s="202"/>
-      <c r="M29" s="203"/>
+      <c r="J29" s="192"/>
+      <c r="K29" s="192"/>
+      <c r="L29" s="192"/>
+      <c r="M29" s="190"/>
       <c r="N29" s="28"/>
       <c r="O29" s="28"/>
       <c r="P29" s="28"/>
@@ -4644,22 +4644,22 @@
     <row r="31" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="32" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="33" spans="2:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="204" t="s">
+      <c r="B33" s="199" t="s">
         <v>48</v>
       </c>
       <c r="C33" s="20"/>
-      <c r="D33" s="206" t="s">
+      <c r="D33" s="201" t="s">
         <v>49</v>
       </c>
-      <c r="E33" s="207"/>
+      <c r="E33" s="202"/>
     </row>
     <row r="34" spans="2:5" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="205"/>
+      <c r="B34" s="200"/>
       <c r="C34" s="24"/>
-      <c r="D34" s="208" t="s">
+      <c r="D34" s="203" t="s">
         <v>50</v>
       </c>
-      <c r="E34" s="207"/>
+      <c r="E34" s="202"/>
     </row>
     <row r="35" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="36" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -5629,13 +5629,11 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="B16:B18"/>
+    <mergeCell ref="C16:D18"/>
+    <mergeCell ref="E16:K16"/>
     <mergeCell ref="L16:M16"/>
     <mergeCell ref="B24:D24"/>
     <mergeCell ref="B25:D25"/>
@@ -5645,11 +5643,13 @@
     <mergeCell ref="D34:E34"/>
     <mergeCell ref="I28:M28"/>
     <mergeCell ref="I29:M29"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="B16:B18"/>
-    <mergeCell ref="C16:D18"/>
-    <mergeCell ref="E16:K16"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D8:E8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup scale="69" orientation="landscape"/>
@@ -5663,39 +5663,39 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="4" spans="1:1" ht="17.25" x14ac:dyDescent="0.25">
-      <c r="A4" s="323" t="s">
+      <c r="A4" s="184" t="s">
         <v>251</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="324"/>
+      <c r="A5" s="185"/>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="325" t="s">
+      <c r="A6" s="186" t="s">
         <v>252</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="324"/>
+      <c r="A7" s="185"/>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="325" t="s">
+      <c r="A8" s="186" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="324"/>
+      <c r="A9" s="185"/>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="325" t="s">
+      <c r="A10" s="186" t="s">
         <v>254</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="324"/>
+      <c r="A11" s="185"/>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" s="325" t="s">
+      <c r="A12" s="186" t="s">
         <v>255</v>
       </c>
     </row>
@@ -5727,38 +5727,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="21.75" x14ac:dyDescent="0.35">
-      <c r="A1" s="237" t="s">
+      <c r="A1" s="223" t="s">
         <v>51</v>
       </c>
-      <c r="B1" s="207"/>
-      <c r="C1" s="207"/>
-      <c r="D1" s="207"/>
-      <c r="E1" s="207"/>
-      <c r="F1" s="207"/>
-      <c r="G1" s="207"/>
-      <c r="H1" s="207"/>
-      <c r="I1" s="207"/>
-      <c r="J1" s="207"/>
-      <c r="K1" s="207"/>
+      <c r="B1" s="202"/>
+      <c r="C1" s="202"/>
+      <c r="D1" s="202"/>
+      <c r="E1" s="202"/>
+      <c r="F1" s="202"/>
+      <c r="G1" s="202"/>
+      <c r="H1" s="202"/>
+      <c r="I1" s="202"/>
+      <c r="J1" s="202"/>
+      <c r="K1" s="202"/>
       <c r="L1" s="6"/>
       <c r="M1" s="6"/>
       <c r="N1" s="6"/>
       <c r="O1" s="6"/>
     </row>
     <row r="2" spans="1:15" ht="21.75" x14ac:dyDescent="0.35">
-      <c r="A2" s="237" t="s">
+      <c r="A2" s="223" t="s">
         <v>52</v>
       </c>
-      <c r="B2" s="207"/>
-      <c r="C2" s="207"/>
-      <c r="D2" s="207"/>
-      <c r="E2" s="207"/>
-      <c r="F2" s="207"/>
-      <c r="G2" s="207"/>
-      <c r="H2" s="207"/>
-      <c r="I2" s="207"/>
-      <c r="J2" s="207"/>
-      <c r="K2" s="207"/>
+      <c r="B2" s="202"/>
+      <c r="C2" s="202"/>
+      <c r="D2" s="202"/>
+      <c r="E2" s="202"/>
+      <c r="F2" s="202"/>
+      <c r="G2" s="202"/>
+      <c r="H2" s="202"/>
+      <c r="I2" s="202"/>
+      <c r="J2" s="202"/>
+      <c r="K2" s="202"/>
       <c r="L2" s="6"/>
       <c r="M2" s="6"/>
       <c r="N2" s="6"/>
@@ -5769,11 +5769,11 @@
       <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="238" t="str">
+      <c r="C3" s="224" t="str">
         <f>'PO Set Target attain level'!D3</f>
         <v>SEMINAR AND PROJECT INITIATION COURSE</v>
       </c>
-      <c r="D3" s="185"/>
+      <c r="D3" s="188"/>
       <c r="E3" s="6"/>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
@@ -5791,11 +5791,11 @@
       <c r="B4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="238">
+      <c r="C4" s="224">
         <f>'PO Set Target attain level'!D4</f>
         <v>315003</v>
       </c>
-      <c r="D4" s="185"/>
+      <c r="D4" s="188"/>
       <c r="E4" s="6"/>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
@@ -5813,11 +5813,11 @@
       <c r="B5" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C5" s="238" t="str">
+      <c r="C5" s="224" t="str">
         <f>'PO Set Target attain level'!D5</f>
         <v>5th Sem Co5K K-Scheme</v>
       </c>
-      <c r="D5" s="185"/>
+      <c r="D5" s="188"/>
       <c r="E5" s="6"/>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
@@ -5835,11 +5835,11 @@
       <c r="B6" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="C6" s="238" t="str">
+      <c r="C6" s="224" t="str">
         <f>'PO Set Target attain level'!D6</f>
         <v>2025-26</v>
       </c>
-      <c r="D6" s="185"/>
+      <c r="D6" s="188"/>
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
@@ -5870,31 +5870,31 @@
       <c r="O7" s="6"/>
     </row>
     <row r="8" spans="1:15" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="239" t="s">
+      <c r="A8" s="225" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="216" t="s">
+      <c r="B8" s="249" t="s">
         <v>55</v>
       </c>
-      <c r="C8" s="217" t="s">
+      <c r="C8" s="250" t="s">
         <v>56</v>
       </c>
-      <c r="D8" s="233" t="s">
+      <c r="D8" s="253" t="s">
         <v>57</v>
       </c>
-      <c r="E8" s="234" t="s">
+      <c r="E8" s="254" t="s">
         <v>58</v>
       </c>
-      <c r="F8" s="212" t="s">
+      <c r="F8" s="247" t="s">
         <v>59</v>
       </c>
-      <c r="G8" s="215" t="s">
+      <c r="G8" s="248" t="s">
         <v>60</v>
       </c>
-      <c r="H8" s="235" t="s">
+      <c r="H8" s="219" t="s">
         <v>61</v>
       </c>
-      <c r="I8" s="236" t="s">
+      <c r="I8" s="222" t="s">
         <v>62</v>
       </c>
       <c r="J8" s="29" t="s">
@@ -5909,62 +5909,62 @@
       <c r="O8" s="6"/>
     </row>
     <row r="9" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="213"/>
-      <c r="B9" s="213"/>
-      <c r="C9" s="213"/>
-      <c r="D9" s="213"/>
-      <c r="E9" s="213"/>
-      <c r="F9" s="213"/>
-      <c r="G9" s="213"/>
-      <c r="H9" s="213"/>
-      <c r="I9" s="213"/>
-      <c r="J9" s="240" t="s">
+      <c r="A9" s="220"/>
+      <c r="B9" s="220"/>
+      <c r="C9" s="220"/>
+      <c r="D9" s="220"/>
+      <c r="E9" s="220"/>
+      <c r="F9" s="220"/>
+      <c r="G9" s="220"/>
+      <c r="H9" s="220"/>
+      <c r="I9" s="220"/>
+      <c r="J9" s="226" t="s">
         <v>65</v>
       </c>
-      <c r="K9" s="241"/>
+      <c r="K9" s="227"/>
       <c r="L9" s="6"/>
       <c r="M9" s="6"/>
       <c r="N9" s="6"/>
       <c r="O9" s="6"/>
     </row>
     <row r="10" spans="1:15" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="213"/>
-      <c r="B10" s="213"/>
-      <c r="C10" s="213"/>
-      <c r="D10" s="213"/>
-      <c r="E10" s="213"/>
-      <c r="F10" s="213"/>
-      <c r="G10" s="213"/>
-      <c r="H10" s="213"/>
-      <c r="I10" s="213"/>
-      <c r="J10" s="242"/>
-      <c r="K10" s="205"/>
+      <c r="A10" s="220"/>
+      <c r="B10" s="220"/>
+      <c r="C10" s="220"/>
+      <c r="D10" s="220"/>
+      <c r="E10" s="220"/>
+      <c r="F10" s="220"/>
+      <c r="G10" s="220"/>
+      <c r="H10" s="220"/>
+      <c r="I10" s="220"/>
+      <c r="J10" s="228"/>
+      <c r="K10" s="200"/>
       <c r="L10" s="6"/>
       <c r="M10" s="6"/>
       <c r="N10" s="6"/>
       <c r="O10" s="6"/>
     </row>
     <row r="11" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="213"/>
-      <c r="B11" s="213"/>
-      <c r="C11" s="213"/>
-      <c r="D11" s="214"/>
-      <c r="E11" s="214"/>
-      <c r="F11" s="214"/>
-      <c r="G11" s="214"/>
-      <c r="H11" s="214"/>
-      <c r="I11" s="214"/>
-      <c r="J11" s="243"/>
-      <c r="K11" s="244"/>
+      <c r="A11" s="220"/>
+      <c r="B11" s="220"/>
+      <c r="C11" s="220"/>
+      <c r="D11" s="221"/>
+      <c r="E11" s="221"/>
+      <c r="F11" s="221"/>
+      <c r="G11" s="221"/>
+      <c r="H11" s="221"/>
+      <c r="I11" s="221"/>
+      <c r="J11" s="229"/>
+      <c r="K11" s="230"/>
       <c r="L11" s="6"/>
       <c r="M11" s="6"/>
       <c r="N11" s="6"/>
       <c r="O11" s="6"/>
     </row>
     <row r="12" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="214"/>
-      <c r="B12" s="214"/>
-      <c r="C12" s="214"/>
+      <c r="A12" s="221"/>
+      <c r="B12" s="221"/>
+      <c r="C12" s="221"/>
       <c r="D12" s="30">
         <v>8</v>
       </c>
@@ -8324,93 +8324,93 @@
       <c r="O95" s="6"/>
     </row>
     <row r="96" spans="1:15" ht="60.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A96" s="218" t="s">
+      <c r="A96" s="251" t="s">
         <v>129</v>
       </c>
-      <c r="B96" s="207"/>
+      <c r="B96" s="202"/>
       <c r="C96" s="40">
         <v>0.4</v>
       </c>
-      <c r="D96" s="219">
+      <c r="D96" s="215">
         <f t="shared" ref="D96:I96" si="2">$C$96*D12</f>
         <v>3.2</v>
       </c>
-      <c r="E96" s="219">
+      <c r="E96" s="215">
         <f t="shared" si="2"/>
         <v>4.8000000000000007</v>
       </c>
-      <c r="F96" s="219">
+      <c r="F96" s="215">
         <f t="shared" si="2"/>
         <v>3.2</v>
       </c>
-      <c r="G96" s="219">
+      <c r="G96" s="215">
         <f t="shared" si="2"/>
         <v>3.2</v>
       </c>
-      <c r="H96" s="219">
+      <c r="H96" s="215">
         <f t="shared" si="2"/>
         <v>4.8000000000000007</v>
       </c>
-      <c r="I96" s="219">
+      <c r="I96" s="215">
         <f t="shared" si="2"/>
         <v>3.2</v>
       </c>
-      <c r="J96" s="245"/>
-      <c r="K96" s="245"/>
+      <c r="J96" s="216"/>
+      <c r="K96" s="216"/>
       <c r="L96" s="6"/>
       <c r="M96" s="6"/>
       <c r="N96" s="6"/>
       <c r="O96" s="6"/>
     </row>
     <row r="97" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A97" s="220" t="s">
+      <c r="A97" s="252" t="s">
         <v>130</v>
       </c>
-      <c r="B97" s="207"/>
-      <c r="C97" s="192"/>
-      <c r="D97" s="188"/>
-      <c r="E97" s="188"/>
-      <c r="F97" s="188"/>
-      <c r="G97" s="188"/>
-      <c r="H97" s="188"/>
-      <c r="I97" s="188"/>
-      <c r="J97" s="188"/>
-      <c r="K97" s="188"/>
+      <c r="B97" s="202"/>
+      <c r="C97" s="211"/>
+      <c r="D97" s="207"/>
+      <c r="E97" s="207"/>
+      <c r="F97" s="207"/>
+      <c r="G97" s="207"/>
+      <c r="H97" s="207"/>
+      <c r="I97" s="207"/>
+      <c r="J97" s="207"/>
+      <c r="K97" s="207"/>
       <c r="L97" s="6"/>
       <c r="M97" s="6"/>
       <c r="N97" s="6"/>
       <c r="O97" s="6"/>
     </row>
     <row r="98" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A98" s="207"/>
-      <c r="B98" s="207"/>
-      <c r="C98" s="192"/>
-      <c r="D98" s="247">
+      <c r="A98" s="202"/>
+      <c r="B98" s="202"/>
+      <c r="C98" s="211"/>
+      <c r="D98" s="218">
         <f t="shared" ref="D98:I98" si="3">COUNTIF(D13:D95,"&gt;=" &amp;D96)</f>
         <v>0</v>
       </c>
-      <c r="E98" s="247">
+      <c r="E98" s="218">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="F98" s="247">
+      <c r="F98" s="218">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="G98" s="247">
+      <c r="G98" s="218">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="H98" s="247">
+      <c r="H98" s="218">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="I98" s="247">
+      <c r="I98" s="218">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="J98" s="246"/>
-      <c r="K98" s="246"/>
+      <c r="J98" s="217"/>
+      <c r="K98" s="217"/>
       <c r="L98" s="6"/>
       <c r="M98" s="6"/>
       <c r="N98" s="6"/>
@@ -8420,14 +8420,14 @@
       <c r="A99" s="6"/>
       <c r="B99" s="6"/>
       <c r="C99" s="6"/>
-      <c r="D99" s="188"/>
-      <c r="E99" s="188"/>
-      <c r="F99" s="188"/>
-      <c r="G99" s="188"/>
-      <c r="H99" s="188"/>
-      <c r="I99" s="188"/>
-      <c r="J99" s="188"/>
-      <c r="K99" s="188"/>
+      <c r="D99" s="207"/>
+      <c r="E99" s="207"/>
+      <c r="F99" s="207"/>
+      <c r="G99" s="207"/>
+      <c r="H99" s="207"/>
+      <c r="I99" s="207"/>
+      <c r="J99" s="207"/>
+      <c r="K99" s="207"/>
       <c r="L99" s="6"/>
       <c r="M99" s="6"/>
       <c r="N99" s="6"/>
@@ -8486,21 +8486,21 @@
     </row>
     <row r="103" spans="1:15" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="6"/>
-      <c r="B103" s="226" t="s">
+      <c r="B103" s="236" t="s">
         <v>131</v>
       </c>
       <c r="C103" s="196"/>
       <c r="D103" s="196"/>
-      <c r="E103" s="197"/>
-      <c r="F103" s="227" t="s">
+      <c r="E103" s="194"/>
+      <c r="F103" s="237" t="s">
         <v>132</v>
       </c>
-      <c r="G103" s="197"/>
+      <c r="G103" s="194"/>
       <c r="H103" s="41"/>
-      <c r="I103" s="228" t="s">
+      <c r="I103" s="238" t="s">
         <v>133</v>
       </c>
-      <c r="J103" s="197"/>
+      <c r="J103" s="194"/>
       <c r="K103" s="6"/>
       <c r="L103" s="6"/>
       <c r="M103" s="6"/>
@@ -8509,28 +8509,28 @@
     </row>
     <row r="104" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="6"/>
-      <c r="B104" s="229" t="s">
+      <c r="B104" s="239" t="s">
         <v>134</v>
       </c>
-      <c r="C104" s="221" t="s">
+      <c r="C104" s="231" t="s">
         <v>135</v>
       </c>
-      <c r="D104" s="222"/>
+      <c r="D104" s="232"/>
       <c r="E104" s="42">
         <v>50</v>
       </c>
-      <c r="F104" s="232">
+      <c r="F104" s="242">
         <v>63</v>
       </c>
-      <c r="G104" s="190"/>
+      <c r="G104" s="209"/>
       <c r="H104" s="43">
         <f>E104*F104/100</f>
         <v>31.5</v>
       </c>
-      <c r="I104" s="248">
+      <c r="I104" s="243">
         <v>1</v>
       </c>
-      <c r="J104" s="249"/>
+      <c r="J104" s="244"/>
       <c r="K104" s="6"/>
       <c r="L104" s="6"/>
       <c r="M104" s="6"/>
@@ -8539,24 +8539,24 @@
     </row>
     <row r="105" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="6"/>
-      <c r="B105" s="230"/>
-      <c r="C105" s="221" t="s">
+      <c r="B105" s="240"/>
+      <c r="C105" s="231" t="s">
         <v>136</v>
       </c>
-      <c r="D105" s="222"/>
+      <c r="D105" s="232"/>
       <c r="E105" s="42">
         <v>60</v>
       </c>
-      <c r="F105" s="191"/>
-      <c r="G105" s="192"/>
+      <c r="F105" s="210"/>
+      <c r="G105" s="211"/>
       <c r="H105" s="44">
         <f>E105*F104/100</f>
         <v>37.799999999999997</v>
       </c>
-      <c r="I105" s="250">
+      <c r="I105" s="245">
         <v>2</v>
       </c>
-      <c r="J105" s="251"/>
+      <c r="J105" s="246"/>
       <c r="K105" s="6"/>
       <c r="L105" s="6"/>
       <c r="M105" s="6"/>
@@ -8565,24 +8565,24 @@
     </row>
     <row r="106" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="6"/>
-      <c r="B106" s="231"/>
-      <c r="C106" s="221" t="s">
+      <c r="B106" s="241"/>
+      <c r="C106" s="231" t="s">
         <v>137</v>
       </c>
-      <c r="D106" s="222"/>
+      <c r="D106" s="232"/>
       <c r="E106" s="45">
         <v>70</v>
       </c>
-      <c r="F106" s="193"/>
-      <c r="G106" s="194"/>
+      <c r="F106" s="212"/>
+      <c r="G106" s="213"/>
       <c r="H106" s="46">
         <f>E106*F104/100</f>
         <v>44.1</v>
       </c>
-      <c r="I106" s="223">
+      <c r="I106" s="233">
         <v>3</v>
       </c>
-      <c r="J106" s="224"/>
+      <c r="J106" s="234"/>
       <c r="K106" s="6"/>
       <c r="L106" s="6"/>
       <c r="M106" s="6"/>
@@ -8597,9 +8597,9 @@
       <c r="E107" s="47"/>
       <c r="F107" s="47"/>
       <c r="G107" s="47"/>
-      <c r="H107" s="225"/>
-      <c r="I107" s="202"/>
-      <c r="J107" s="203"/>
+      <c r="H107" s="235"/>
+      <c r="I107" s="192"/>
+      <c r="J107" s="190"/>
       <c r="K107" s="6"/>
       <c r="L107" s="6"/>
       <c r="M107" s="6"/>
@@ -8614,9 +8614,9 @@
       <c r="E108" s="47"/>
       <c r="F108" s="47"/>
       <c r="G108" s="47"/>
-      <c r="H108" s="225"/>
-      <c r="I108" s="202"/>
-      <c r="J108" s="203"/>
+      <c r="H108" s="235"/>
+      <c r="I108" s="192"/>
+      <c r="J108" s="190"/>
       <c r="K108" s="6"/>
       <c r="L108" s="6"/>
       <c r="M108" s="6"/>
@@ -12961,24 +12961,16 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="H96:H97"/>
-    <mergeCell ref="I96:I97"/>
-    <mergeCell ref="J96:J97"/>
-    <mergeCell ref="K96:K97"/>
-    <mergeCell ref="J98:J99"/>
-    <mergeCell ref="K98:K99"/>
-    <mergeCell ref="H98:H99"/>
-    <mergeCell ref="I98:I99"/>
-    <mergeCell ref="H8:H11"/>
-    <mergeCell ref="I8:I11"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="A8:A12"/>
-    <mergeCell ref="J9:K11"/>
+    <mergeCell ref="A96:B96"/>
+    <mergeCell ref="E96:E97"/>
+    <mergeCell ref="F96:F97"/>
+    <mergeCell ref="G96:G97"/>
+    <mergeCell ref="A97:C98"/>
+    <mergeCell ref="D96:D97"/>
+    <mergeCell ref="D98:D99"/>
+    <mergeCell ref="E98:E99"/>
+    <mergeCell ref="F98:F99"/>
+    <mergeCell ref="G98:G99"/>
     <mergeCell ref="C106:D106"/>
     <mergeCell ref="I106:J106"/>
     <mergeCell ref="H107:J107"/>
@@ -12992,22 +12984,30 @@
     <mergeCell ref="C105:D105"/>
     <mergeCell ref="I104:J104"/>
     <mergeCell ref="I105:J105"/>
+    <mergeCell ref="H8:H11"/>
+    <mergeCell ref="I8:I11"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="A8:A12"/>
+    <mergeCell ref="J9:K11"/>
     <mergeCell ref="F8:F11"/>
     <mergeCell ref="G8:G11"/>
     <mergeCell ref="B8:B12"/>
     <mergeCell ref="C8:C12"/>
-    <mergeCell ref="A96:B96"/>
-    <mergeCell ref="E96:E97"/>
-    <mergeCell ref="F96:F97"/>
-    <mergeCell ref="G96:G97"/>
-    <mergeCell ref="A97:C98"/>
     <mergeCell ref="D8:D11"/>
     <mergeCell ref="E8:E11"/>
-    <mergeCell ref="D96:D97"/>
-    <mergeCell ref="D98:D99"/>
-    <mergeCell ref="E98:E99"/>
-    <mergeCell ref="F98:F99"/>
-    <mergeCell ref="G98:G99"/>
+    <mergeCell ref="H96:H97"/>
+    <mergeCell ref="I96:I97"/>
+    <mergeCell ref="J96:J97"/>
+    <mergeCell ref="K96:K97"/>
+    <mergeCell ref="J98:J99"/>
+    <mergeCell ref="K98:K99"/>
+    <mergeCell ref="H98:H99"/>
+    <mergeCell ref="I98:I99"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -13033,13 +13033,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:22" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="B1" s="252" t="s">
+      <c r="B1" s="267" t="s">
         <v>143</v>
       </c>
-      <c r="C1" s="207"/>
-      <c r="D1" s="207"/>
-      <c r="E1" s="207"/>
-      <c r="F1" s="207"/>
+      <c r="C1" s="202"/>
+      <c r="D1" s="202"/>
+      <c r="E1" s="202"/>
+      <c r="F1" s="202"/>
       <c r="G1" s="6"/>
       <c r="H1" s="6"/>
       <c r="I1" s="6"/>
@@ -13108,11 +13108,11 @@
       <c r="C4" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="253" t="str">
+      <c r="D4" s="268" t="str">
         <f>'CO_Attainment for Unit Tests'!C3</f>
         <v>SEMINAR AND PROJECT INITIATION COURSE</v>
       </c>
-      <c r="E4" s="203"/>
+      <c r="E4" s="190"/>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
       <c r="H4" s="6"/>
@@ -13136,11 +13136,11 @@
       <c r="C5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="253">
+      <c r="D5" s="268">
         <f>'CO_Attainment for Unit Tests'!C4</f>
         <v>315003</v>
       </c>
-      <c r="E5" s="203"/>
+      <c r="E5" s="190"/>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
@@ -13164,11 +13164,11 @@
       <c r="C6" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D6" s="253" t="str">
+      <c r="D6" s="268" t="str">
         <f>'CO_Attainment for Unit Tests'!C5</f>
         <v>5th Sem Co5K K-Scheme</v>
       </c>
-      <c r="E6" s="203"/>
+      <c r="E6" s="190"/>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
       <c r="H6" s="6"/>
@@ -13192,11 +13192,11 @@
       <c r="C7" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="253" t="str">
+      <c r="D7" s="268" t="str">
         <f>'CO_Attainment for Unit Tests'!C6</f>
         <v>2025-26</v>
       </c>
-      <c r="E7" s="203"/>
+      <c r="E7" s="190"/>
       <c r="F7" s="6"/>
       <c r="G7" s="6"/>
       <c r="H7" s="6"/>
@@ -13219,41 +13219,41 @@
       <c r="E8" s="10"/>
     </row>
     <row r="9" spans="2:22" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="254" t="s">
+      <c r="B9" s="262" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="255" t="s">
+      <c r="C9" s="257" t="s">
         <v>55</v>
       </c>
-      <c r="D9" s="217" t="s">
+      <c r="D9" s="250" t="s">
         <v>56</v>
       </c>
-      <c r="E9" s="255" t="s">
+      <c r="E9" s="257" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="10" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B10" s="213"/>
-      <c r="C10" s="213"/>
-      <c r="D10" s="213"/>
-      <c r="E10" s="213"/>
+      <c r="B10" s="220"/>
+      <c r="C10" s="220"/>
+      <c r="D10" s="220"/>
+      <c r="E10" s="220"/>
     </row>
     <row r="11" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B11" s="213"/>
-      <c r="C11" s="213"/>
-      <c r="D11" s="213"/>
-      <c r="E11" s="213"/>
+      <c r="B11" s="220"/>
+      <c r="C11" s="220"/>
+      <c r="D11" s="220"/>
+      <c r="E11" s="220"/>
     </row>
     <row r="12" spans="2:22" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="213"/>
-      <c r="C12" s="213"/>
-      <c r="D12" s="213"/>
-      <c r="E12" s="214"/>
+      <c r="B12" s="220"/>
+      <c r="C12" s="220"/>
+      <c r="D12" s="220"/>
+      <c r="E12" s="221"/>
     </row>
     <row r="13" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B13" s="214"/>
-      <c r="C13" s="214"/>
-      <c r="D13" s="214"/>
+      <c r="B13" s="221"/>
+      <c r="C13" s="221"/>
+      <c r="D13" s="221"/>
       <c r="E13" s="54">
         <v>70</v>
       </c>
@@ -14426,7 +14426,7 @@
       <c r="D97" s="57" t="s">
         <v>146</v>
       </c>
-      <c r="E97" s="262">
+      <c r="E97" s="258">
         <f>D98*E13/100</f>
         <v>32.878999999999998</v>
       </c>
@@ -14435,7 +14435,7 @@
       <c r="D98" s="58">
         <v>46.97</v>
       </c>
-      <c r="E98" s="188"/>
+      <c r="E98" s="207"/>
     </row>
     <row r="99" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D99" s="59" t="s">
@@ -14461,12 +14461,12 @@
       <c r="E102" s="10"/>
     </row>
     <row r="103" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A103" s="226" t="s">
+      <c r="A103" s="236" t="s">
         <v>131</v>
       </c>
       <c r="B103" s="196"/>
       <c r="C103" s="196"/>
-      <c r="D103" s="197"/>
+      <c r="D103" s="194"/>
       <c r="E103" s="63" t="s">
         <v>132</v>
       </c>
@@ -14478,17 +14478,17 @@
       <c r="I103" s="65"/>
     </row>
     <row r="104" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A104" s="229" t="s">
+      <c r="A104" s="239" t="s">
         <v>134</v>
       </c>
       <c r="B104" s="66">
         <v>0.5</v>
       </c>
-      <c r="C104" s="263" t="s">
+      <c r="C104" s="259" t="s">
         <v>148</v>
       </c>
-      <c r="D104" s="264"/>
-      <c r="E104" s="265">
+      <c r="D104" s="260"/>
+      <c r="E104" s="261">
         <f>COUNTA(D14:D96)-COUNTIFS(D14:D96,0)</f>
         <v>63</v>
       </c>
@@ -14503,15 +14503,15 @@
       <c r="I104" s="65"/>
     </row>
     <row r="105" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A105" s="230"/>
+      <c r="A105" s="240"/>
       <c r="B105" s="69">
         <v>0.6</v>
       </c>
-      <c r="C105" s="256" t="s">
+      <c r="C105" s="263" t="s">
         <v>148</v>
       </c>
-      <c r="D105" s="251"/>
-      <c r="E105" s="187"/>
+      <c r="D105" s="246"/>
+      <c r="E105" s="206"/>
       <c r="F105" s="70">
         <f t="shared" si="0"/>
         <v>37.799999999999997</v>
@@ -14523,15 +14523,15 @@
       <c r="I105" s="65"/>
     </row>
     <row r="106" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A106" s="231"/>
+      <c r="A106" s="241"/>
       <c r="B106" s="72">
         <v>0.7</v>
       </c>
-      <c r="C106" s="257" t="s">
+      <c r="C106" s="264" t="s">
         <v>149</v>
       </c>
-      <c r="D106" s="224"/>
-      <c r="E106" s="188"/>
+      <c r="D106" s="234"/>
+      <c r="E106" s="207"/>
       <c r="F106" s="73">
         <f t="shared" si="0"/>
         <v>44.099999999999994</v>
@@ -14565,10 +14565,10 @@
       <c r="I108" s="65"/>
     </row>
     <row r="109" spans="1:9" ht="71.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A109" s="258" t="s">
+      <c r="A109" s="265" t="s">
         <v>150</v>
       </c>
-      <c r="B109" s="259"/>
+      <c r="B109" s="266"/>
       <c r="C109" s="49" t="s">
         <v>9</v>
       </c>
@@ -14590,10 +14590,10 @@
       <c r="I109" s="65"/>
     </row>
     <row r="110" spans="1:9" ht="39" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A110" s="260" t="s">
+      <c r="A110" s="255" t="s">
         <v>151</v>
       </c>
-      <c r="B110" s="261"/>
+      <c r="B110" s="256"/>
       <c r="C110" s="52">
         <f>IF(E99&gt;=$F106,3,IF(E99&gt;=$F105,2,IF(E99&gt;=$F104,1,0)))</f>
         <v>0</v>
@@ -15932,6 +15932,11 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="B1:F1"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
     <mergeCell ref="A110:B110"/>
     <mergeCell ref="D9:D13"/>
     <mergeCell ref="E9:E12"/>
@@ -15945,11 +15950,6 @@
     <mergeCell ref="C105:D105"/>
     <mergeCell ref="C106:D106"/>
     <mergeCell ref="A109:B109"/>
-    <mergeCell ref="B1:F1"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="portrait"/>
@@ -16006,11 +16006,11 @@
       <c r="C4" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="238" t="str">
+      <c r="D4" s="224" t="str">
         <f>'CO_Attainment for Unit Tests'!C3</f>
         <v>SEMINAR AND PROJECT INITIATION COURSE</v>
       </c>
-      <c r="E4" s="185"/>
+      <c r="E4" s="188"/>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
       <c r="H4" s="6"/>
@@ -16020,11 +16020,11 @@
       <c r="C5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="238">
+      <c r="D5" s="224">
         <f>'CO_Attainment for Unit Tests'!C4</f>
         <v>315003</v>
       </c>
-      <c r="E5" s="185"/>
+      <c r="E5" s="188"/>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
@@ -16034,11 +16034,11 @@
       <c r="C6" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="D6" s="238" t="str">
+      <c r="D6" s="224" t="str">
         <f>'CO_Attainment for Unit Tests'!C5</f>
         <v>5th Sem Co5K K-Scheme</v>
       </c>
-      <c r="E6" s="185"/>
+      <c r="E6" s="188"/>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
       <c r="H6" s="6"/>
@@ -16048,63 +16048,63 @@
       <c r="C7" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="D7" s="238" t="str">
+      <c r="D7" s="224" t="str">
         <f>'CO_Attainment for Unit Tests'!C6</f>
         <v>2025-26</v>
       </c>
-      <c r="E7" s="185"/>
+      <c r="E7" s="188"/>
       <c r="F7" s="6"/>
       <c r="G7" s="6"/>
       <c r="H7" s="6"/>
     </row>
     <row r="9" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="254" t="s">
+      <c r="B9" s="262" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="255" t="s">
+      <c r="C9" s="257" t="s">
         <v>55</v>
       </c>
-      <c r="D9" s="266" t="s">
+      <c r="D9" s="274" t="s">
         <v>56</v>
       </c>
-      <c r="E9" s="255" t="s">
+      <c r="E9" s="257" t="s">
         <v>156</v>
       </c>
-      <c r="F9" s="255" t="s">
+      <c r="F9" s="257" t="s">
         <v>157</v>
       </c>
-      <c r="G9" s="255" t="s">
+      <c r="G9" s="257" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="10" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="213"/>
-      <c r="C10" s="213"/>
-      <c r="D10" s="213"/>
-      <c r="E10" s="213"/>
-      <c r="F10" s="213"/>
-      <c r="G10" s="213"/>
+      <c r="B10" s="220"/>
+      <c r="C10" s="220"/>
+      <c r="D10" s="220"/>
+      <c r="E10" s="220"/>
+      <c r="F10" s="220"/>
+      <c r="G10" s="220"/>
     </row>
     <row r="11" spans="2:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="213"/>
-      <c r="C11" s="213"/>
-      <c r="D11" s="213"/>
-      <c r="E11" s="213"/>
-      <c r="F11" s="213"/>
-      <c r="G11" s="213"/>
+      <c r="B11" s="220"/>
+      <c r="C11" s="220"/>
+      <c r="D11" s="220"/>
+      <c r="E11" s="220"/>
+      <c r="F11" s="220"/>
+      <c r="G11" s="220"/>
     </row>
     <row r="12" spans="2:8" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="213"/>
-      <c r="C12" s="213"/>
-      <c r="D12" s="213"/>
-      <c r="E12" s="214"/>
-      <c r="F12" s="214"/>
-      <c r="G12" s="214"/>
+      <c r="B12" s="220"/>
+      <c r="C12" s="220"/>
+      <c r="D12" s="220"/>
+      <c r="E12" s="221"/>
+      <c r="F12" s="221"/>
+      <c r="G12" s="221"/>
     </row>
     <row r="13" spans="2:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="214"/>
-      <c r="C13" s="214"/>
-      <c r="D13" s="214"/>
+      <c r="B13" s="221"/>
+      <c r="C13" s="221"/>
+      <c r="D13" s="221"/>
       <c r="E13" s="32">
         <v>25</v>
       </c>
@@ -17827,15 +17827,15 @@
       <c r="D97" s="81" t="s">
         <v>159</v>
       </c>
-      <c r="E97" s="267">
+      <c r="E97" s="270">
         <f>ROUNDUP(D98*E13/100,1)</f>
         <v>15</v>
       </c>
-      <c r="F97" s="267">
+      <c r="F97" s="270">
         <f>ROUNDUP(D98*F13/100,1)</f>
         <v>15</v>
       </c>
-      <c r="G97" s="267">
+      <c r="G97" s="270">
         <f>ROUNDUP(D98*G13/100,1)</f>
         <v>15</v>
       </c>
@@ -17844,9 +17844,9 @@
       <c r="D98" s="82">
         <v>60</v>
       </c>
-      <c r="E98" s="188"/>
-      <c r="F98" s="188"/>
-      <c r="G98" s="188"/>
+      <c r="E98" s="207"/>
+      <c r="F98" s="207"/>
+      <c r="G98" s="207"/>
     </row>
     <row r="99" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D99" s="59" t="s">
@@ -17870,11 +17870,11 @@
     <row r="102" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="103" spans="1:8" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="65"/>
-      <c r="B103" s="226" t="s">
+      <c r="B103" s="236" t="s">
         <v>160</v>
       </c>
       <c r="C103" s="196"/>
-      <c r="D103" s="197"/>
+      <c r="D103" s="194"/>
       <c r="E103" s="83" t="s">
         <v>132</v>
       </c>
@@ -17886,7 +17886,7 @@
     </row>
     <row r="104" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="65"/>
-      <c r="B104" s="229" t="s">
+      <c r="B104" s="239" t="s">
         <v>134</v>
       </c>
       <c r="C104" s="66">
@@ -17895,7 +17895,7 @@
       <c r="D104" s="67" t="s">
         <v>149</v>
       </c>
-      <c r="E104" s="265">
+      <c r="E104" s="261">
         <f>COUNTA(D14:D96)-COUNTIFS(D14:D96,0)</f>
         <v>63</v>
       </c>
@@ -17910,14 +17910,14 @@
     </row>
     <row r="105" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="65"/>
-      <c r="B105" s="230"/>
+      <c r="B105" s="240"/>
       <c r="C105" s="69">
         <v>0.6</v>
       </c>
       <c r="D105" s="70" t="s">
         <v>149</v>
       </c>
-      <c r="E105" s="187"/>
+      <c r="E105" s="206"/>
       <c r="F105" s="85">
         <f>C105*$E104</f>
         <v>37.799999999999997</v>
@@ -17929,14 +17929,14 @@
     </row>
     <row r="106" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="65"/>
-      <c r="B106" s="231"/>
+      <c r="B106" s="241"/>
       <c r="C106" s="72">
         <v>0.7</v>
       </c>
       <c r="D106" s="73" t="s">
         <v>149</v>
       </c>
-      <c r="E106" s="188"/>
+      <c r="E106" s="207"/>
       <c r="F106" s="86">
         <f>C106*$E104</f>
         <v>44.099999999999994</v>
@@ -17967,10 +17967,10 @@
       <c r="H108" s="65"/>
     </row>
     <row r="109" spans="1:8" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A109" s="195" t="s">
+      <c r="A109" s="214" t="s">
         <v>161</v>
       </c>
-      <c r="B109" s="268"/>
+      <c r="B109" s="271"/>
       <c r="C109" s="87" t="s">
         <v>9</v>
       </c>
@@ -17991,10 +17991,10 @@
       </c>
     </row>
     <row r="110" spans="1:8" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A110" s="269" t="s">
+      <c r="A110" s="272" t="s">
         <v>162</v>
       </c>
-      <c r="B110" s="259"/>
+      <c r="B110" s="266"/>
       <c r="C110" s="89">
         <f>IF(E99&gt;=$F106,3,IF(E99&gt;=$F105,2,IF(E99&gt;=$F104,1,0)))</f>
         <v>3</v>
@@ -18021,10 +18021,10 @@
       </c>
     </row>
     <row r="111" spans="1:8" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A111" s="270" t="s">
+      <c r="A111" s="273" t="s">
         <v>163</v>
       </c>
-      <c r="B111" s="185"/>
+      <c r="B111" s="188"/>
       <c r="C111" s="91">
         <f>IF(F99&gt;=$F106,3,IF(F99&gt;=$F105,2,IF(F99&gt;=$F104,1,0)))</f>
         <v>3</v>
@@ -18051,10 +18051,10 @@
       </c>
     </row>
     <row r="112" spans="1:8" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A112" s="271" t="s">
+      <c r="A112" s="269" t="s">
         <v>164</v>
       </c>
-      <c r="B112" s="261"/>
+      <c r="B112" s="256"/>
       <c r="C112" s="52">
         <f>IF(G99&gt;=$F106,3,IF(G99&gt;=$F105,2,IF(G99&gt;=$F104,1,0)))</f>
         <v>3</v>
@@ -18980,6 +18980,13 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="B9:B13"/>
+    <mergeCell ref="C9:C13"/>
+    <mergeCell ref="D9:D13"/>
     <mergeCell ref="A112:B112"/>
     <mergeCell ref="E9:E12"/>
     <mergeCell ref="F9:F12"/>
@@ -18993,13 +19000,6 @@
     <mergeCell ref="A109:B109"/>
     <mergeCell ref="A110:B110"/>
     <mergeCell ref="A111:B111"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="B9:B13"/>
-    <mergeCell ref="C9:C13"/>
-    <mergeCell ref="D9:D13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup scale="28" orientation="landscape"/>
@@ -19101,41 +19101,41 @@
       </c>
     </row>
     <row r="10" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="278" t="s">
+      <c r="B10" s="287" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="279" t="s">
+      <c r="C10" s="275" t="s">
         <v>167</v>
       </c>
-      <c r="D10" s="280" t="s">
+      <c r="D10" s="288" t="s">
         <v>56</v>
       </c>
-      <c r="E10" s="279" t="s">
+      <c r="E10" s="275" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B11" s="187"/>
-      <c r="C11" s="187"/>
-      <c r="D11" s="187"/>
-      <c r="E11" s="187"/>
+      <c r="B11" s="206"/>
+      <c r="C11" s="206"/>
+      <c r="D11" s="206"/>
+      <c r="E11" s="206"/>
     </row>
     <row r="12" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B12" s="187"/>
-      <c r="C12" s="187"/>
-      <c r="D12" s="187"/>
-      <c r="E12" s="187"/>
+      <c r="B12" s="206"/>
+      <c r="C12" s="206"/>
+      <c r="D12" s="206"/>
+      <c r="E12" s="206"/>
     </row>
     <row r="13" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B13" s="187"/>
-      <c r="C13" s="187"/>
-      <c r="D13" s="187"/>
-      <c r="E13" s="281"/>
+      <c r="B13" s="206"/>
+      <c r="C13" s="206"/>
+      <c r="D13" s="206"/>
+      <c r="E13" s="276"/>
     </row>
     <row r="14" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B14" s="188"/>
-      <c r="C14" s="188"/>
-      <c r="D14" s="188"/>
+      <c r="B14" s="207"/>
+      <c r="C14" s="207"/>
+      <c r="D14" s="207"/>
       <c r="E14" s="96">
         <v>5</v>
       </c>
@@ -19932,57 +19932,57 @@
     </row>
     <row r="84" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="85" spans="1:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="282" t="s">
+      <c r="A85" s="277" t="s">
         <v>173</v>
       </c>
       <c r="B85" s="196"/>
       <c r="C85" s="196"/>
-      <c r="D85" s="197"/>
+      <c r="D85" s="194"/>
       <c r="E85" s="103" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="86" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="283" t="s">
+      <c r="A86" s="278" t="s">
         <v>134</v>
       </c>
-      <c r="B86" s="284" t="s">
+      <c r="B86" s="279" t="s">
         <v>174</v>
       </c>
-      <c r="C86" s="285"/>
-      <c r="D86" s="264"/>
+      <c r="C86" s="280"/>
+      <c r="D86" s="260"/>
       <c r="E86" s="104">
         <v>1</v>
       </c>
     </row>
     <row r="87" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="230"/>
-      <c r="B87" s="272" t="s">
+      <c r="A87" s="240"/>
+      <c r="B87" s="281" t="s">
         <v>175</v>
       </c>
-      <c r="C87" s="273"/>
-      <c r="D87" s="251"/>
+      <c r="C87" s="282"/>
+      <c r="D87" s="246"/>
       <c r="E87" s="105">
         <v>2</v>
       </c>
     </row>
     <row r="88" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A88" s="231"/>
-      <c r="B88" s="274" t="s">
+      <c r="A88" s="241"/>
+      <c r="B88" s="283" t="s">
         <v>176</v>
       </c>
-      <c r="C88" s="275"/>
-      <c r="D88" s="224"/>
+      <c r="C88" s="284"/>
+      <c r="D88" s="234"/>
       <c r="E88" s="106">
         <v>3</v>
       </c>
     </row>
     <row r="89" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="90" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A90" s="276" t="s">
+      <c r="A90" s="285" t="s">
         <v>161</v>
       </c>
-      <c r="B90" s="268"/>
+      <c r="B90" s="271"/>
       <c r="C90" s="107" t="s">
         <v>9</v>
       </c>
@@ -20000,10 +20000,10 @@
       </c>
     </row>
     <row r="91" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A91" s="277" t="s">
+      <c r="A91" s="286" t="s">
         <v>177</v>
       </c>
-      <c r="B91" s="259"/>
+      <c r="B91" s="266"/>
       <c r="C91" s="109">
         <f>IF(E81&gt;=80,3,IF(E81&gt;=65,2,IF(E81&gt;=40,1,0)))</f>
         <v>0</v>
@@ -20945,17 +20945,17 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="A90:B90"/>
+    <mergeCell ref="A91:B91"/>
+    <mergeCell ref="B10:B14"/>
+    <mergeCell ref="C10:C14"/>
+    <mergeCell ref="D10:D14"/>
     <mergeCell ref="E10:E13"/>
     <mergeCell ref="A85:D85"/>
     <mergeCell ref="A86:A88"/>
     <mergeCell ref="B86:D86"/>
     <mergeCell ref="B87:D87"/>
     <mergeCell ref="B88:D88"/>
-    <mergeCell ref="A90:B90"/>
-    <mergeCell ref="A91:B91"/>
-    <mergeCell ref="B10:B14"/>
-    <mergeCell ref="C10:C14"/>
-    <mergeCell ref="D10:D14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="portrait"/>
@@ -21020,14 +21020,14 @@
       <c r="P5" s="10"/>
     </row>
     <row r="6" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B6" s="186" t="s">
+      <c r="B6" s="205" t="s">
         <v>21</v>
       </c>
-      <c r="C6" s="189" t="s">
+      <c r="C6" s="208" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="190"/>
-      <c r="E6" s="195" t="s">
+      <c r="D6" s="209"/>
+      <c r="E6" s="214" t="s">
         <v>23</v>
       </c>
       <c r="F6" s="196"/>
@@ -21038,16 +21038,16 @@
       <c r="K6" s="196"/>
       <c r="L6" s="196"/>
       <c r="M6" s="196"/>
-      <c r="N6" s="197"/>
-      <c r="O6" s="195" t="s">
+      <c r="N6" s="194"/>
+      <c r="O6" s="214" t="s">
         <v>24</v>
       </c>
-      <c r="P6" s="197"/>
+      <c r="P6" s="194"/>
     </row>
     <row r="7" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B7" s="187"/>
-      <c r="C7" s="191"/>
-      <c r="D7" s="192"/>
+      <c r="B7" s="206"/>
+      <c r="C7" s="210"/>
+      <c r="D7" s="211"/>
       <c r="E7" s="13" t="s">
         <v>25</v>
       </c>
@@ -21086,9 +21086,9 @@
       </c>
     </row>
     <row r="8" spans="2:16" ht="62.25" x14ac:dyDescent="0.25">
-      <c r="B8" s="188"/>
-      <c r="C8" s="193"/>
-      <c r="D8" s="194"/>
+      <c r="B8" s="207"/>
+      <c r="C8" s="212"/>
+      <c r="D8" s="213"/>
       <c r="E8" s="15" t="s">
         <v>186</v>
       </c>
@@ -21409,11 +21409,11 @@
       </c>
     </row>
     <row r="15" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B15" s="286" t="s">
+      <c r="B15" s="290" t="s">
         <v>205</v>
       </c>
       <c r="C15" s="196"/>
-      <c r="D15" s="197"/>
+      <c r="D15" s="194"/>
       <c r="E15" s="116">
         <f t="shared" ref="E15:P15" si="0">ROUNDUP(AVERAGE(E9:E14),2)</f>
         <v>3</v>
@@ -21464,11 +21464,11 @@
       </c>
     </row>
     <row r="16" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B16" s="287" t="s">
+      <c r="B16" s="289" t="s">
         <v>206</v>
       </c>
       <c r="C16" s="196"/>
-      <c r="D16" s="197"/>
+      <c r="D16" s="194"/>
       <c r="E16" s="117">
         <f t="shared" ref="E16:P16" si="1">ROUNDUP((E15*2.66)/3,2)</f>
         <v>2.66</v>
@@ -21519,11 +21519,11 @@
       </c>
     </row>
     <row r="17" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B17" s="287" t="s">
+      <c r="B17" s="289" t="s">
         <v>207</v>
       </c>
       <c r="C17" s="196"/>
-      <c r="D17" s="197"/>
+      <c r="D17" s="194"/>
       <c r="E17" s="117">
         <f t="shared" ref="E17:P17" si="2">ROUNDUP((E16/3)*100,2)</f>
         <v>88.67</v>
@@ -22555,13 +22555,13 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="7">
+    <mergeCell ref="O6:P6"/>
+    <mergeCell ref="B15:D15"/>
     <mergeCell ref="B16:D16"/>
     <mergeCell ref="B17:D17"/>
     <mergeCell ref="B6:B8"/>
     <mergeCell ref="C6:D8"/>
     <mergeCell ref="E6:N6"/>
-    <mergeCell ref="O6:P6"/>
-    <mergeCell ref="B15:D15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -22810,7 +22810,7 @@
     <row r="8" spans="1:26" ht="21" x14ac:dyDescent="0.25">
       <c r="A8" s="10"/>
       <c r="B8" s="10"/>
-      <c r="C8" s="288" t="s">
+      <c r="C8" s="297" t="s">
         <v>209</v>
       </c>
       <c r="D8" s="196"/>
@@ -22819,7 +22819,7 @@
       <c r="G8" s="196"/>
       <c r="H8" s="196"/>
       <c r="I8" s="196"/>
-      <c r="J8" s="197"/>
+      <c r="J8" s="194"/>
       <c r="K8" s="10"/>
       <c r="L8" s="10"/>
       <c r="M8" s="10"/>
@@ -22840,18 +22840,18 @@
     <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A9" s="10"/>
       <c r="B9" s="10"/>
-      <c r="C9" s="289" t="s">
+      <c r="C9" s="298" t="s">
         <v>210</v>
       </c>
       <c r="D9" s="196"/>
       <c r="E9" s="196"/>
       <c r="F9" s="196"/>
       <c r="G9" s="196"/>
-      <c r="H9" s="197"/>
-      <c r="I9" s="290" t="s">
+      <c r="H9" s="194"/>
+      <c r="I9" s="299" t="s">
         <v>211</v>
       </c>
-      <c r="J9" s="190"/>
+      <c r="J9" s="209"/>
       <c r="K9" s="10"/>
       <c r="L9" s="10"/>
       <c r="M9" s="10"/>
@@ -22872,20 +22872,20 @@
     <row r="10" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A10" s="10"/>
       <c r="B10" s="10"/>
-      <c r="C10" s="291" t="s">
+      <c r="C10" s="300" t="s">
         <v>212</v>
       </c>
-      <c r="D10" s="292" t="s">
+      <c r="D10" s="301" t="s">
         <v>213</v>
       </c>
-      <c r="E10" s="293"/>
-      <c r="F10" s="293"/>
-      <c r="G10" s="194"/>
+      <c r="E10" s="302"/>
+      <c r="F10" s="302"/>
+      <c r="G10" s="213"/>
       <c r="H10" s="119" t="s">
         <v>214</v>
       </c>
-      <c r="I10" s="193"/>
-      <c r="J10" s="194"/>
+      <c r="I10" s="212"/>
+      <c r="J10" s="213"/>
       <c r="K10" s="10"/>
       <c r="L10" s="10"/>
       <c r="M10" s="10"/>
@@ -22906,7 +22906,7 @@
     <row r="11" spans="1:26" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="10"/>
       <c r="B11" s="10"/>
-      <c r="C11" s="188"/>
+      <c r="C11" s="207"/>
       <c r="D11" s="120" t="s">
         <v>215</v>
       </c>
@@ -22922,10 +22922,10 @@
       <c r="H11" s="123" t="s">
         <v>219</v>
       </c>
-      <c r="I11" s="294" t="s">
+      <c r="I11" s="303" t="s">
         <v>220</v>
       </c>
-      <c r="J11" s="197"/>
+      <c r="J11" s="194"/>
       <c r="K11" s="10"/>
       <c r="L11" s="10"/>
       <c r="M11" s="10"/>
@@ -22969,11 +22969,11 @@
         <f>'CO_attainment for FA-TH ESE'!C110</f>
         <v>0</v>
       </c>
-      <c r="I12" s="295">
+      <c r="I12" s="293">
         <f>'CO_attainment for Indirect'!C91</f>
         <v>0</v>
       </c>
-      <c r="J12" s="264"/>
+      <c r="J12" s="260"/>
       <c r="K12" s="10"/>
       <c r="L12" s="10"/>
       <c r="M12" s="10"/>
@@ -23017,11 +23017,11 @@
         <f t="shared" ref="H13:H17" si="3">$H12</f>
         <v>0</v>
       </c>
-      <c r="I13" s="299">
+      <c r="I13" s="292">
         <f t="shared" ref="I13:I17" si="4">$I12</f>
         <v>0</v>
       </c>
-      <c r="J13" s="251"/>
+      <c r="J13" s="246"/>
       <c r="K13" s="10"/>
       <c r="L13" s="10"/>
       <c r="M13" s="10"/>
@@ -23065,11 +23065,11 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="I14" s="299">
+      <c r="I14" s="292">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="J14" s="251"/>
+      <c r="J14" s="246"/>
       <c r="K14" s="10"/>
       <c r="L14" s="10"/>
       <c r="M14" s="10"/>
@@ -23113,11 +23113,11 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="I15" s="299">
+      <c r="I15" s="292">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="J15" s="251"/>
+      <c r="J15" s="246"/>
       <c r="K15" s="10"/>
       <c r="L15" s="10"/>
       <c r="M15" s="10"/>
@@ -23161,11 +23161,11 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="I16" s="299">
+      <c r="I16" s="292">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="J16" s="251"/>
+      <c r="J16" s="246"/>
       <c r="K16" s="10"/>
       <c r="L16" s="10"/>
       <c r="M16" s="10"/>
@@ -23209,11 +23209,11 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="I17" s="299">
+      <c r="I17" s="292">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="J17" s="251"/>
+      <c r="J17" s="246"/>
       <c r="K17" s="10"/>
       <c r="L17" s="10"/>
       <c r="M17" s="10"/>
@@ -23257,11 +23257,11 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="I18" s="295">
+      <c r="I18" s="293">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="J18" s="264"/>
+      <c r="J18" s="260"/>
       <c r="K18" s="10"/>
       <c r="L18" s="10"/>
       <c r="M18" s="10"/>
@@ -23300,10 +23300,10 @@
       <c r="H19" s="137">
         <v>60</v>
       </c>
-      <c r="I19" s="300">
+      <c r="I19" s="294">
         <v>100</v>
       </c>
-      <c r="J19" s="185"/>
+      <c r="J19" s="188"/>
       <c r="K19" s="10"/>
       <c r="L19" s="10"/>
       <c r="M19" s="10"/>
@@ -23347,11 +23347,11 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="I20" s="296">
+      <c r="I20" s="295">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="J20" s="224"/>
+      <c r="J20" s="234"/>
       <c r="K20" s="10"/>
       <c r="L20" s="10"/>
       <c r="M20" s="10"/>
@@ -23372,13 +23372,13 @@
     <row r="21" spans="1:26" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="10"/>
       <c r="B21" s="10"/>
-      <c r="C21" s="297" t="s">
+      <c r="C21" s="296" t="s">
         <v>224</v>
       </c>
       <c r="D21" s="196"/>
       <c r="E21" s="196"/>
       <c r="F21" s="196"/>
-      <c r="G21" s="197"/>
+      <c r="G21" s="194"/>
       <c r="H21" s="139">
         <f>SUM(D20:H20)</f>
         <v>0.89999999999999991</v>
@@ -23410,13 +23410,13 @@
     <row r="22" spans="1:26" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="10"/>
       <c r="B22" s="10"/>
-      <c r="C22" s="297" t="s">
+      <c r="C22" s="296" t="s">
         <v>226</v>
       </c>
       <c r="D22" s="196"/>
       <c r="E22" s="196"/>
       <c r="F22" s="196"/>
-      <c r="G22" s="197"/>
+      <c r="G22" s="194"/>
       <c r="H22" s="141">
         <v>0.8</v>
       </c>
@@ -23446,13 +23446,13 @@
     <row r="23" spans="1:26" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="10"/>
       <c r="B23" s="10"/>
-      <c r="C23" s="297" t="s">
+      <c r="C23" s="296" t="s">
         <v>228</v>
       </c>
       <c r="D23" s="196"/>
       <c r="E23" s="196"/>
       <c r="F23" s="196"/>
-      <c r="G23" s="197"/>
+      <c r="G23" s="194"/>
       <c r="H23" s="139">
         <f>0.8*H21</f>
         <v>0.72</v>
@@ -23484,14 +23484,14 @@
     <row r="24" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="10"/>
       <c r="B24" s="10"/>
-      <c r="C24" s="298" t="s">
+      <c r="C24" s="291" t="s">
         <v>230</v>
       </c>
       <c r="D24" s="196"/>
       <c r="E24" s="196"/>
       <c r="F24" s="196"/>
       <c r="G24" s="196"/>
-      <c r="H24" s="197"/>
+      <c r="H24" s="194"/>
       <c r="I24" s="143">
         <f>ROUNDUP(H23+J23,2)</f>
         <v>0.72</v>
@@ -30085,6 +30085,17 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="C8:J8"/>
+    <mergeCell ref="C9:H9"/>
+    <mergeCell ref="I9:J10"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="D10:G10"/>
+    <mergeCell ref="I11:J11"/>
+    <mergeCell ref="I12:J12"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="C21:G21"/>
+    <mergeCell ref="C22:G22"/>
+    <mergeCell ref="C23:G23"/>
     <mergeCell ref="C24:H24"/>
     <mergeCell ref="I13:J13"/>
     <mergeCell ref="I14:J14"/>
@@ -30093,17 +30104,6 @@
     <mergeCell ref="I17:J17"/>
     <mergeCell ref="I18:J18"/>
     <mergeCell ref="I19:J19"/>
-    <mergeCell ref="I12:J12"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="C21:G21"/>
-    <mergeCell ref="C22:G22"/>
-    <mergeCell ref="C23:G23"/>
-    <mergeCell ref="C8:J8"/>
-    <mergeCell ref="C9:H9"/>
-    <mergeCell ref="I9:J10"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="D10:G10"/>
-    <mergeCell ref="I11:J11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="portrait"/>
@@ -30353,15 +30353,15 @@
     <row r="8" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A8" s="10"/>
       <c r="B8" s="6"/>
-      <c r="C8" s="301" t="s">
+      <c r="C8" s="318" t="s">
         <v>233</v>
       </c>
-      <c r="D8" s="302"/>
-      <c r="E8" s="304" t="s">
+      <c r="D8" s="319"/>
+      <c r="E8" s="321" t="s">
         <v>234</v>
       </c>
-      <c r="F8" s="285"/>
-      <c r="G8" s="259"/>
+      <c r="F8" s="280"/>
+      <c r="G8" s="266"/>
       <c r="H8" s="145" t="s">
         <v>235</v>
       </c>
@@ -30371,7 +30371,7 @@
       <c r="J8" s="145" t="s">
         <v>237</v>
       </c>
-      <c r="K8" s="305" t="s">
+      <c r="K8" s="322" t="s">
         <v>238</v>
       </c>
       <c r="L8" s="10"/>
@@ -30393,8 +30393,8 @@
     <row r="9" spans="1:26" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="10"/>
       <c r="B9" s="6"/>
-      <c r="C9" s="193"/>
-      <c r="D9" s="303"/>
+      <c r="C9" s="212"/>
+      <c r="D9" s="320"/>
       <c r="E9" s="146" t="s">
         <v>239</v>
       </c>
@@ -30413,7 +30413,7 @@
       <c r="J9" s="147" t="s">
         <v>219</v>
       </c>
-      <c r="K9" s="306"/>
+      <c r="K9" s="323"/>
       <c r="L9" s="10"/>
       <c r="M9" s="10"/>
       <c r="N9" s="10"/>
@@ -30433,14 +30433,14 @@
     <row r="10" spans="1:26" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="10"/>
       <c r="B10" s="6"/>
-      <c r="C10" s="307" t="s">
+      <c r="C10" s="324" t="s">
         <v>243</v>
       </c>
-      <c r="D10" s="259"/>
-      <c r="E10" s="308">
+      <c r="D10" s="266"/>
+      <c r="E10" s="325">
         <v>0</v>
       </c>
-      <c r="F10" s="259"/>
+      <c r="F10" s="266"/>
       <c r="G10" s="148">
         <v>25</v>
       </c>
@@ -30476,15 +30476,15 @@
     <row r="11" spans="1:26" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="10"/>
       <c r="B11" s="6"/>
-      <c r="C11" s="309" t="s">
+      <c r="C11" s="311" t="s">
         <v>244</v>
       </c>
-      <c r="D11" s="261"/>
-      <c r="E11" s="310">
+      <c r="D11" s="256"/>
+      <c r="E11" s="312">
         <f>(E10/$K10)*100</f>
         <v>0</v>
       </c>
-      <c r="F11" s="261"/>
+      <c r="F11" s="256"/>
       <c r="G11" s="149">
         <f t="shared" ref="G11:J11" si="1">(G10/$K10)*100</f>
         <v>33.333333333333329</v>
@@ -30608,7 +30608,7 @@
     <row r="15" spans="1:26" ht="21" x14ac:dyDescent="0.25">
       <c r="A15" s="10"/>
       <c r="B15" s="10"/>
-      <c r="C15" s="311" t="s">
+      <c r="C15" s="313" t="s">
         <v>209</v>
       </c>
       <c r="D15" s="196"/>
@@ -30617,7 +30617,7 @@
       <c r="G15" s="196"/>
       <c r="H15" s="196"/>
       <c r="I15" s="196"/>
-      <c r="J15" s="197"/>
+      <c r="J15" s="194"/>
       <c r="K15" s="10"/>
       <c r="L15" s="10"/>
       <c r="M15" s="10"/>
@@ -30638,16 +30638,16 @@
     <row r="16" spans="1:26" ht="21" x14ac:dyDescent="0.25">
       <c r="A16" s="10"/>
       <c r="B16" s="10"/>
-      <c r="C16" s="312" t="s">
+      <c r="C16" s="314" t="s">
         <v>210</v>
       </c>
       <c r="D16" s="196"/>
       <c r="E16" s="196"/>
       <c r="F16" s="196"/>
       <c r="G16" s="196"/>
-      <c r="H16" s="197"/>
-      <c r="I16" s="313"/>
-      <c r="J16" s="190"/>
+      <c r="H16" s="194"/>
+      <c r="I16" s="315"/>
+      <c r="J16" s="209"/>
       <c r="K16" s="10"/>
       <c r="L16" s="10"/>
       <c r="M16" s="10"/>
@@ -30668,7 +30668,7 @@
     <row r="17" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A17" s="10"/>
       <c r="B17" s="10"/>
-      <c r="C17" s="314" t="s">
+      <c r="C17" s="316" t="s">
         <v>245</v>
       </c>
       <c r="D17" s="151"/>
@@ -30680,8 +30680,8 @@
       <c r="H17" s="155" t="s">
         <v>214</v>
       </c>
-      <c r="I17" s="193"/>
-      <c r="J17" s="194"/>
+      <c r="I17" s="212"/>
+      <c r="J17" s="213"/>
       <c r="K17" s="10"/>
       <c r="L17" s="10"/>
       <c r="M17" s="10"/>
@@ -30702,7 +30702,7 @@
     <row r="18" spans="1:26" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="10"/>
       <c r="B18" s="10"/>
-      <c r="C18" s="188"/>
+      <c r="C18" s="207"/>
       <c r="D18" s="156" t="s">
         <v>215</v>
       </c>
@@ -30718,8 +30718,8 @@
       <c r="H18" s="159" t="s">
         <v>219</v>
       </c>
-      <c r="I18" s="315"/>
-      <c r="J18" s="197"/>
+      <c r="I18" s="317"/>
+      <c r="J18" s="194"/>
       <c r="K18" s="10"/>
       <c r="L18" s="10"/>
       <c r="M18" s="10"/>
@@ -30763,8 +30763,8 @@
         <f>'CO_attainment for FA-TH ESE'!C110</f>
         <v>0</v>
       </c>
-      <c r="I19" s="316"/>
-      <c r="J19" s="264"/>
+      <c r="I19" s="307"/>
+      <c r="J19" s="260"/>
       <c r="K19" s="10"/>
       <c r="L19" s="10"/>
       <c r="M19" s="10"/>
@@ -30808,8 +30808,8 @@
         <f t="shared" ref="H20:H24" si="5">$H19</f>
         <v>0</v>
       </c>
-      <c r="I20" s="317"/>
-      <c r="J20" s="251"/>
+      <c r="I20" s="306"/>
+      <c r="J20" s="246"/>
       <c r="K20" s="10"/>
       <c r="L20" s="10"/>
       <c r="M20" s="10"/>
@@ -30853,8 +30853,8 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="I21" s="317"/>
-      <c r="J21" s="251"/>
+      <c r="I21" s="306"/>
+      <c r="J21" s="246"/>
       <c r="K21" s="10"/>
       <c r="L21" s="10"/>
       <c r="M21" s="10"/>
@@ -30898,8 +30898,8 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="I22" s="317"/>
-      <c r="J22" s="251"/>
+      <c r="I22" s="306"/>
+      <c r="J22" s="246"/>
       <c r="K22" s="10"/>
       <c r="L22" s="10"/>
       <c r="M22" s="10"/>
@@ -30943,8 +30943,8 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="I23" s="317"/>
-      <c r="J23" s="251"/>
+      <c r="I23" s="306"/>
+      <c r="J23" s="246"/>
       <c r="K23" s="10"/>
       <c r="L23" s="10"/>
       <c r="M23" s="10"/>
@@ -30988,8 +30988,8 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="I24" s="317"/>
-      <c r="J24" s="251"/>
+      <c r="I24" s="306"/>
+      <c r="J24" s="246"/>
       <c r="K24" s="10"/>
       <c r="L24" s="10"/>
       <c r="M24" s="10"/>
@@ -31033,8 +31033,8 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="I25" s="316"/>
-      <c r="J25" s="264"/>
+      <c r="I25" s="307"/>
+      <c r="J25" s="260"/>
       <c r="K25" s="10"/>
       <c r="L25" s="10"/>
       <c r="M25" s="10"/>
@@ -31078,8 +31078,8 @@
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
-      <c r="I26" s="321"/>
-      <c r="J26" s="251"/>
+      <c r="I26" s="308"/>
+      <c r="J26" s="246"/>
       <c r="K26" s="10"/>
       <c r="L26" s="10"/>
       <c r="M26" s="10"/>
@@ -31123,8 +31123,8 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="I27" s="322"/>
-      <c r="J27" s="224"/>
+      <c r="I27" s="309"/>
+      <c r="J27" s="234"/>
       <c r="K27" s="10"/>
       <c r="L27" s="10"/>
       <c r="M27" s="10"/>
@@ -31145,13 +31145,13 @@
     <row r="28" spans="1:26" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="10"/>
       <c r="B28" s="10"/>
-      <c r="C28" s="318" t="s">
+      <c r="C28" s="310" t="s">
         <v>224</v>
       </c>
       <c r="D28" s="196"/>
       <c r="E28" s="196"/>
       <c r="F28" s="196"/>
-      <c r="G28" s="197"/>
+      <c r="G28" s="194"/>
       <c r="H28" s="174">
         <f>SUM(D27:H27)</f>
         <v>2.9999999999999996</v>
@@ -31178,13 +31178,13 @@
     <row r="29" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="10"/>
       <c r="B29" s="10"/>
-      <c r="C29" s="318" t="s">
+      <c r="C29" s="310" t="s">
         <v>226</v>
       </c>
       <c r="D29" s="196"/>
       <c r="E29" s="196"/>
       <c r="F29" s="196"/>
-      <c r="G29" s="197"/>
+      <c r="G29" s="194"/>
       <c r="H29" s="177">
         <v>1</v>
       </c>
@@ -31210,13 +31210,13 @@
     <row r="30" spans="1:26" ht="62.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="10"/>
       <c r="B30" s="10"/>
-      <c r="C30" s="318" t="s">
+      <c r="C30" s="310" t="s">
         <v>228</v>
       </c>
       <c r="D30" s="196"/>
       <c r="E30" s="196"/>
       <c r="F30" s="196"/>
-      <c r="G30" s="197"/>
+      <c r="G30" s="194"/>
       <c r="H30" s="174">
         <f>H29*H28</f>
         <v>2.9999999999999996</v>
@@ -31243,14 +31243,14 @@
     <row r="31" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="10"/>
       <c r="B31" s="10"/>
-      <c r="C31" s="319" t="s">
+      <c r="C31" s="304" t="s">
         <v>230</v>
       </c>
       <c r="D31" s="196"/>
       <c r="E31" s="196"/>
       <c r="F31" s="196"/>
       <c r="G31" s="196"/>
-      <c r="H31" s="197"/>
+      <c r="H31" s="194"/>
       <c r="I31" s="179">
         <f>H30+J30</f>
         <v>2.9999999999999996</v>
@@ -31337,11 +31337,11 @@
       <c r="E34" s="10"/>
       <c r="F34" s="10"/>
       <c r="G34" s="10"/>
-      <c r="H34" s="209" t="s">
+      <c r="H34" s="204" t="s">
         <v>46</v>
       </c>
-      <c r="I34" s="207"/>
-      <c r="J34" s="207"/>
+      <c r="I34" s="202"/>
+      <c r="J34" s="202"/>
       <c r="L34" s="10"/>
       <c r="M34" s="10"/>
       <c r="N34" s="10"/>
@@ -31366,11 +31366,11 @@
       <c r="E35" s="10"/>
       <c r="F35" s="10"/>
       <c r="G35" s="10"/>
-      <c r="H35" s="320" t="s">
+      <c r="H35" s="305" t="s">
         <v>47</v>
       </c>
-      <c r="I35" s="202"/>
-      <c r="J35" s="203"/>
+      <c r="I35" s="192"/>
+      <c r="J35" s="190"/>
       <c r="K35" s="11"/>
       <c r="L35" s="11"/>
       <c r="M35" s="11"/>
@@ -37755,6 +37755,23 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="27">
+    <mergeCell ref="C8:D9"/>
+    <mergeCell ref="E8:G8"/>
+    <mergeCell ref="K8:K9"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="C15:J15"/>
+    <mergeCell ref="C16:H16"/>
+    <mergeCell ref="I16:J17"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="I18:J18"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="C28:G28"/>
+    <mergeCell ref="C29:G29"/>
+    <mergeCell ref="C30:G30"/>
     <mergeCell ref="C31:H31"/>
     <mergeCell ref="H34:J34"/>
     <mergeCell ref="H35:J35"/>
@@ -37765,23 +37782,6 @@
     <mergeCell ref="I25:J25"/>
     <mergeCell ref="I26:J26"/>
     <mergeCell ref="I27:J27"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="C28:G28"/>
-    <mergeCell ref="C29:G29"/>
-    <mergeCell ref="C30:G30"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="C15:J15"/>
-    <mergeCell ref="C16:H16"/>
-    <mergeCell ref="I16:J17"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="I18:J18"/>
-    <mergeCell ref="C8:D9"/>
-    <mergeCell ref="E8:G8"/>
-    <mergeCell ref="K8:K9"/>
-    <mergeCell ref="C10:D10"/>
-    <mergeCell ref="E10:F10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -37846,11 +37846,11 @@
       <c r="C2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="238" t="str">
+      <c r="D2" s="224" t="str">
         <f>'Overall CO attainment'!D3</f>
         <v>SEMINAR AND PROJECT INITIATION COURSE</v>
       </c>
-      <c r="E2" s="185"/>
+      <c r="E2" s="188"/>
       <c r="F2" s="11"/>
       <c r="G2" s="11"/>
       <c r="H2" s="11"/>
@@ -37878,11 +37878,11 @@
       <c r="C3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="238">
+      <c r="D3" s="224">
         <f>'Overall CO attainment'!D4</f>
         <v>315003</v>
       </c>
-      <c r="E3" s="185"/>
+      <c r="E3" s="188"/>
       <c r="F3" s="11"/>
       <c r="G3" s="11"/>
       <c r="H3" s="11"/>
@@ -37910,11 +37910,11 @@
       <c r="C4" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="238" t="str">
+      <c r="D4" s="224" t="str">
         <f>'Overall CO attainment'!D5</f>
         <v>5th Sem Co5K K-Scheme</v>
       </c>
-      <c r="E4" s="185"/>
+      <c r="E4" s="188"/>
       <c r="F4" s="11"/>
       <c r="G4" s="11"/>
       <c r="H4" s="11"/>
@@ -37942,11 +37942,11 @@
       <c r="C5" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="D5" s="238" t="str">
+      <c r="D5" s="224" t="str">
         <f>'Overall CO attainment'!D6</f>
         <v>2025-26</v>
       </c>
-      <c r="E5" s="185"/>
+      <c r="E5" s="188"/>
       <c r="F5" s="11"/>
       <c r="G5" s="11"/>
       <c r="H5" s="11"/>
@@ -38053,14 +38053,14 @@
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A9" s="11"/>
-      <c r="B9" s="186" t="s">
+      <c r="B9" s="205" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="189" t="s">
+      <c r="C9" s="208" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="190"/>
-      <c r="E9" s="195" t="s">
+      <c r="D9" s="209"/>
+      <c r="E9" s="214" t="s">
         <v>23</v>
       </c>
       <c r="F9" s="196"/>
@@ -38068,11 +38068,11 @@
       <c r="H9" s="196"/>
       <c r="I9" s="196"/>
       <c r="J9" s="196"/>
-      <c r="K9" s="197"/>
-      <c r="L9" s="198" t="s">
+      <c r="K9" s="194"/>
+      <c r="L9" s="193" t="s">
         <v>24</v>
       </c>
-      <c r="M9" s="197"/>
+      <c r="M9" s="194"/>
       <c r="N9" s="11"/>
       <c r="O9" s="11"/>
       <c r="P9" s="11"/>
@@ -38088,9 +38088,9 @@
     </row>
     <row r="10" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11"/>
-      <c r="B10" s="187"/>
-      <c r="C10" s="191"/>
-      <c r="D10" s="192"/>
+      <c r="B10" s="206"/>
+      <c r="C10" s="210"/>
+      <c r="D10" s="211"/>
       <c r="E10" s="13" t="s">
         <v>25</v>
       </c>
@@ -38133,9 +38133,9 @@
     </row>
     <row r="11" spans="1:25" ht="119.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="11"/>
-      <c r="B11" s="188"/>
-      <c r="C11" s="193"/>
-      <c r="D11" s="194"/>
+      <c r="B11" s="207"/>
+      <c r="C11" s="212"/>
+      <c r="D11" s="213"/>
       <c r="E11" s="15" t="s">
         <v>34</v>
       </c>
@@ -38492,11 +38492,11 @@
     </row>
     <row r="17" spans="1:25" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="11"/>
-      <c r="B17" s="199" t="s">
+      <c r="B17" s="195" t="s">
         <v>248</v>
       </c>
       <c r="C17" s="196"/>
-      <c r="D17" s="197"/>
+      <c r="D17" s="194"/>
       <c r="E17" s="18">
         <f t="shared" ref="E17:K17" si="0">IFERROR(AVERAGE(E12:E16),0)</f>
         <v>2.4</v>
@@ -38548,11 +38548,11 @@
     </row>
     <row r="18" spans="1:25" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="11"/>
-      <c r="B18" s="200" t="s">
+      <c r="B18" s="197" t="s">
         <v>249</v>
       </c>
       <c r="C18" s="196"/>
-      <c r="D18" s="197"/>
+      <c r="D18" s="194"/>
       <c r="E18" s="182">
         <f>E17*'Overall CO attainment'!I31/3</f>
         <v>2.3999999999999995</v>
@@ -38604,11 +38604,11 @@
     </row>
     <row r="19" spans="1:25" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="11"/>
-      <c r="B19" s="287" t="s">
+      <c r="B19" s="289" t="s">
         <v>207</v>
       </c>
       <c r="C19" s="196"/>
-      <c r="D19" s="197"/>
+      <c r="D19" s="194"/>
       <c r="E19" s="117">
         <f t="shared" ref="E19:M19" si="3">ROUNDUP((E18/3)*100,2)</f>
         <v>80</v>
@@ -38722,12 +38722,12 @@
       <c r="G22" s="11"/>
       <c r="H22" s="11"/>
       <c r="I22" s="11"/>
-      <c r="J22" s="209" t="s">
+      <c r="J22" s="204" t="s">
         <v>46</v>
       </c>
-      <c r="K22" s="207"/>
-      <c r="L22" s="207"/>
-      <c r="M22" s="207"/>
+      <c r="K22" s="202"/>
+      <c r="L22" s="202"/>
+      <c r="M22" s="202"/>
       <c r="N22" s="11"/>
       <c r="O22" s="11"/>
       <c r="P22" s="11"/>
@@ -38751,12 +38751,12 @@
       <c r="G23" s="11"/>
       <c r="H23" s="11"/>
       <c r="I23" s="11"/>
-      <c r="J23" s="201" t="s">
+      <c r="J23" s="198" t="s">
         <v>47</v>
       </c>
-      <c r="K23" s="202"/>
-      <c r="L23" s="202"/>
-      <c r="M23" s="203"/>
+      <c r="K23" s="192"/>
+      <c r="L23" s="192"/>
+      <c r="M23" s="190"/>
       <c r="N23" s="28"/>
       <c r="O23" s="28"/>
       <c r="P23" s="11"/>
@@ -44949,6 +44949,12 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="B9:B11"/>
+    <mergeCell ref="E9:K9"/>
     <mergeCell ref="L9:M9"/>
     <mergeCell ref="J22:M22"/>
     <mergeCell ref="J23:M23"/>
@@ -44956,12 +44962,6 @@
     <mergeCell ref="B17:D17"/>
     <mergeCell ref="B18:D18"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="D5:E5"/>
-    <mergeCell ref="B9:B11"/>
-    <mergeCell ref="E9:K9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>